<commit_message>
test(oracle): expose criteria intersection gap
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/excel-oracle/criteria-implicit-intersection/fixture.xlsx
+++ b/tests/excel-oracle/criteria-implicit-intersection/fixture.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A298E05-D0AC-4694-89FE-AB7B050175CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F146DF82-9669-436A-BA20-0AC5BE5E9AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{0B715029-B742-4D6E-A093-96A03987E99A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{9BF07AE4-13EB-42F1-BC1B-56B2A200E6EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -414,7 +414,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2A4316C-0D51-46A8-9C9E-AB7379D2902F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{016BB1C7-0765-43C8-BB74-E003133534AA}">
   <dimension ref="E1:P3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -448,7 +448,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E04F7D5E-5CDA-45D5-948E-3F1ACED30AE5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FEB5E5-9A49-48A2-8FD6-3E4883CAC58A}">
   <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>

</xml_diff>

<commit_message>
test(oracle): cover criteria aggregate families
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/excel-oracle/criteria-implicit-intersection/fixture.xlsx
+++ b/tests/excel-oracle/criteria-implicit-intersection/fixture.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F146DF82-9669-436A-BA20-0AC5BE5E9AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A65BFB-DDEA-4A55-8C50-BA469EB27E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{9BF07AE4-13EB-42F1-BC1B-56B2A200E6EE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{016EFE34-9FCD-463F-BB95-9EC25592F274}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -414,7 +414,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{016BB1C7-0765-43C8-BB74-E003133534AA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A4672FC-6C62-489B-B3C2-690D3C74F98F}">
   <dimension ref="E1:P3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -448,11 +448,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FEB5E5-9A49-48A2-8FD6-3E4883CAC58A}">
-  <dimension ref="A1:J15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5BAC412-639A-4698-8EF9-B7637EE81824}">
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B1">
         <v>2</v>
       </c>
@@ -463,8 +463,12 @@
         <f>AVERAGEIF(Data!$E$1:$E$3,$H:$H,Data!$P$1:$P$3)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K1">
+        <f>AVERAGEIFS(Data!$P$1:$P$3,Data!$E$1:$E$3,$H:$H)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="H2" t="s">
         <v>1</v>
       </c>
@@ -472,8 +476,12 @@
         <f>SUMIF(Data!$E$1:$E$3,$H:$H,Data!$P$1:$P$3)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K2">
+        <f>SUMIFS(Data!$P$1:$P$3,Data!$E$1:$E$3,$H:$H)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="H3" t="s">
         <v>2</v>
       </c>
@@ -481,8 +489,12 @@
         <f>COUNTIF(Data!$E$1:$E$3,$H:$H)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K3">
+        <f>COUNTIFS(Data!$E$1:$E$3,$H:$H)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
@@ -493,7 +505,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>10</v>
       </c>
@@ -504,7 +516,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B15">
         <f>SUMIF(A10:C10,1:1,A12:C12)</f>
         <v>20</v>

</xml_diff>

<commit_message>
fix(oracle): normalize case hashes across platforms
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/excel-oracle/criteria-implicit-intersection/fixture.xlsx
+++ b/tests/excel-oracle/criteria-implicit-intersection/fixture.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A65BFB-DDEA-4A55-8C50-BA469EB27E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5122CE-5ADC-422E-B3F8-ACCD29698422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{016EFE34-9FCD-463F-BB95-9EC25592F274}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{CB8C3BB6-F7C9-46FE-9476-BBB9F26ED4F3}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -414,7 +414,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A4672FC-6C62-489B-B3C2-690D3C74F98F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0872C01-62B6-484C-93CB-DF74C9451E42}">
   <dimension ref="E1:P3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -448,7 +448,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5BAC412-639A-4698-8EF9-B7637EE81824}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04C38BD2-A534-410B-AF5A-597742FC0927}">
   <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>

</xml_diff>